<commit_message>
updates the README file, the excel files, Powerquery and PIvot tables
</commit_message>
<xml_diff>
--- a/project/main/template.xlsx
+++ b/project/main/template.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aymeric/Documents/Files_code/excel-project-management/project/main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608E2D8F-1DB6-0048-97BA-99DAC7ECC014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1D8C28-E720-8046-A664-EF3EBC57C071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="2760" windowWidth="27640" windowHeight="16680" xr2:uid="{59A2AF7F-3284-AB42-8105-EDE7504E6F46}"/>
+    <workbookView xWindow="6920" yWindow="2560" windowWidth="27640" windowHeight="16680" xr2:uid="{59A2AF7F-3284-AB42-8105-EDE7504E6F46}"/>
   </bookViews>
   <sheets>
-    <sheet name="Schema" sheetId="1" r:id="rId1"/>
-    <sheet name="Keyword" sheetId="2" r:id="rId2"/>
+    <sheet name="Raw_schema" sheetId="1" r:id="rId1"/>
+    <sheet name="Raw-keywords" sheetId="2" r:id="rId2"/>
+    <sheet name="derivatives-1_schema" sheetId="3" r:id="rId3"/>
+    <sheet name="derivatives-1_keywords" sheetId="4" r:id="rId4"/>
+    <sheet name="derivatives-2_schema" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,10 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="33">
-  <si>
-    <t>File_Type</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="33">
   <si>
     <t>Field</t>
   </si>
@@ -51,24 +51,15 @@
     <t>Data_Type</t>
   </si>
   <si>
-    <t>Required</t>
-  </si>
-  <si>
     <t>Keyword_Group</t>
   </si>
   <si>
-    <t>Experiment</t>
-  </si>
-  <si>
     <t>Experiment_ID</t>
   </si>
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -87,36 +78,18 @@
     <t>Text</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Raw_Data</t>
-  </si>
-  <si>
-    <t>Sample_ID</t>
-  </si>
-  <si>
     <t>Value</t>
   </si>
   <si>
     <t>Number</t>
   </si>
   <si>
-    <t>Derivative1</t>
-  </si>
-  <si>
     <t>Material</t>
   </si>
   <si>
-    <t>Derivative2</t>
-  </si>
-  <si>
     <t>Result</t>
   </si>
   <si>
-    <t>Active</t>
-  </si>
-  <si>
     <t>Planned</t>
   </si>
   <si>
@@ -139,6 +112,36 @@
   </si>
   <si>
     <t>Validation</t>
+  </si>
+  <si>
+    <t>Material_C</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>Explanation</t>
+  </si>
+  <si>
+    <t>correspond to the experiment ID as defined by ABCD</t>
+  </si>
+  <si>
+    <t>Parameter_1</t>
+  </si>
+  <si>
+    <t>Parameter_2</t>
+  </si>
+  <si>
+    <t>Parameter_3</t>
+  </si>
+  <si>
+    <t>Parameters_3</t>
+  </si>
+  <si>
+    <t>Material_D</t>
+  </si>
+  <si>
+    <t>State of the experiment, if it was started or not, if it is ongoing</t>
   </si>
 </sst>
 </file>
@@ -519,10 +522,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A759DDA-A62F-D64B-AC8D-A8F78AB2010D}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -530,190 +536,74 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -723,106 +613,238 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01A9ACED-F74C-984C-BD1D-642B4F03C82C}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF104DBD-5DEB-A844-B609-A32B6E48A8BD}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F0E1C47-6944-3345-B075-ECCC78BE8F2C}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B89166A-51F0-6D4C-AEDA-6C013AD9E7AA}">
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>